<commit_message>
chore: set table names to better values
</commit_message>
<xml_diff>
--- a/src/nist_gas_srm/core/data/template.xlsx
+++ b/src/nist_gas_srm/core/data/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wpk/gits/nist-gas-srm-certificate/nist-gas-srm/src/nist_gas_srm/core/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1ECE6C9-74B2-3F42-98C1-1BE1B85AC2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF043D9-F64D-8743-92B7-2AACAB5312B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2000" yWindow="660" windowWidth="27980" windowHeight="21680" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2000" yWindow="660" windowWidth="27980" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ratio Data" sheetId="1" r:id="rId1"/>
@@ -86,49 +86,6 @@
           </rPr>
           <t>Microsoft Office User:
 = variance / sum(variance)</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Krekelberg, William P. (Fed)</author>
-  </authors>
-  <commentList>
-    <comment ref="U24" authorId="0" shapeId="0" xr:uid="{3A440BC3-64DD-784A-8062-79EA0F3AFF12}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Krekelberg, William P. (Fed):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Fit X-solution vs Y-solution</t>
         </r>
       </text>
     </comment>
@@ -1481,7 +1438,7 @@
     <numFmt numFmtId="178" formatCode="0.0000%"/>
     <numFmt numFmtId="179" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* \-??_);_(@_)"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <name val="Univers"/>
@@ -1649,19 +1606,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -36166,7 +36110,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -37313,7 +37257,6 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToWidth="2" fitToHeight="3" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>